<commit_message>
new matrix algebra doc and update schedule
</commit_message>
<xml_diff>
--- a/comp364-schedule-8-25-2026.xlsx
+++ b/comp364-schedule-8-25-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp364-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63DB3DB-7297-4600-8E7A-0B8A607E4E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2148540F-9F28-4945-A385-838A122E05E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="110">
   <si>
     <t>Class number</t>
   </si>
@@ -466,10 +466,34 @@
     <t>subtopics</t>
   </si>
   <si>
-    <t>Nearest neighbor, using decision tree</t>
-  </si>
-  <si>
     <t>Constructing a decision tree</t>
+  </si>
+  <si>
+    <t>Nearest neighbor; using decision tree</t>
+  </si>
+  <si>
+    <t>Logistic function; Binary cross entropy; SGD for 1D neuron</t>
+  </si>
+  <si>
+    <t>neural nets in PyTorch</t>
+  </si>
+  <si>
+    <t>sustainability (UN SDGs); data center impacts; other sust-AI connections</t>
+  </si>
+  <si>
+    <t>in-class work on posters</t>
+  </si>
+  <si>
+    <t>poster session</t>
+  </si>
+  <si>
+    <t>Turing test; emergence</t>
+  </si>
+  <si>
+    <t>--</t>
+  </si>
+  <si>
+    <t>low-level equivalence of brains and computers; neural networks</t>
   </si>
 </sst>
 </file>
@@ -735,7 +759,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -937,6 +961,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1255,7 +1282,7 @@
     <col min="4" max="4" width="21.28515625" style="7" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" style="6" customWidth="1"/>
+    <col min="7" max="7" width="32.85546875" style="6" customWidth="1"/>
     <col min="8" max="8" width="34.7109375" style="39" customWidth="1"/>
     <col min="9" max="9" width="37.85546875" customWidth="1"/>
   </cols>
@@ -1309,7 +1336,7 @@
       </c>
       <c r="H2" s="34"/>
     </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="50"/>
       <c r="B3" s="16" t="s">
         <v>35</v>
@@ -1373,13 +1400,13 @@
         <v>54</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H5" s="34" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="49">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
@@ -1400,7 +1427,7 @@
         <v>43</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H6" s="34" t="s">
         <v>93</v>
@@ -1423,12 +1450,14 @@
         <v>9</v>
       </c>
       <c r="F7" s="10"/>
-      <c r="G7" s="22"/>
+      <c r="G7" s="22" t="s">
+        <v>107</v>
+      </c>
       <c r="H7" s="34" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="49">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
@@ -1450,7 +1479,9 @@
       <c r="F8" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="22"/>
+      <c r="G8" s="22" t="s">
+        <v>102</v>
+      </c>
       <c r="H8" s="34" t="s">
         <v>95</v>
       </c>
@@ -1472,12 +1503,14 @@
       <c r="F9" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G9" s="22"/>
+      <c r="G9" s="22" t="s">
+        <v>103</v>
+      </c>
       <c r="H9" s="34" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="49">
         <f>A8+1</f>
         <v>5</v>
@@ -1497,12 +1530,14 @@
         <v>12</v>
       </c>
       <c r="F10" s="10"/>
-      <c r="G10" s="22"/>
+      <c r="G10" s="22" t="s">
+        <v>104</v>
+      </c>
       <c r="H10" s="36" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="54"/>
       <c r="B11" s="50"/>
       <c r="C11" s="52"/>
@@ -1531,12 +1566,14 @@
       <c r="F12" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="22"/>
+      <c r="G12" s="22" t="s">
+        <v>105</v>
+      </c>
       <c r="H12" s="34" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="49">
         <f t="shared" ref="A13" si="4">A10+1</f>
         <v>6</v>
@@ -1556,7 +1593,9 @@
       <c r="F13" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="G13" s="22"/>
+      <c r="G13" s="22" t="s">
+        <v>106</v>
+      </c>
       <c r="H13" s="34"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1578,7 +1617,9 @@
       <c r="F14" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="22"/>
+      <c r="G14" s="69" t="s">
+        <v>108</v>
+      </c>
       <c r="H14" s="34"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1601,10 +1642,12 @@
         <v>16</v>
       </c>
       <c r="F15" s="10"/>
-      <c r="G15" s="22"/>
+      <c r="G15" s="69" t="s">
+        <v>108</v>
+      </c>
       <c r="H15" s="35"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="50"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1621,7 +1664,9 @@
         <v>17</v>
       </c>
       <c r="F16" s="10"/>
-      <c r="G16" s="22"/>
+      <c r="G16" s="22" t="s">
+        <v>109</v>
+      </c>
       <c r="H16" s="34" t="s">
         <v>74</v>
       </c>
@@ -1644,7 +1689,7 @@
       <c r="G17" s="42"/>
       <c r="H17" s="34"/>
     </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="49">
         <v>8</v>
       </c>
@@ -1688,7 +1733,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="50"/>
       <c r="B20" s="63"/>
       <c r="C20" s="65"/>
@@ -1700,7 +1745,7 @@
       <c r="G20" s="58"/>
       <c r="H20" s="58"/>
     </row>
-    <row r="21" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="49">
         <v>9</v>
       </c>
@@ -1806,7 +1851,7 @@
       <c r="G25" s="22"/>
       <c r="H25" s="35"/>
     </row>
-    <row r="26" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="59">
         <f>A24+1</f>
         <v>11</v>
@@ -1825,7 +1870,7 @@
       <c r="G26" s="58"/>
       <c r="H26" s="58"/>
     </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="60"/>
       <c r="B27" s="16" t="str">
         <f>B24</f>

</xml_diff>